<commit_message>
chore: actualiza libro excel de entrega y limpia gitignore
</commit_message>
<xml_diff>
--- a/Formatos_Laboratorio_Semana10_Sistema_Matriculas.xlsx
+++ b/Formatos_Laboratorio_Semana10_Sistema_Matriculas.xlsx
@@ -29,39 +29,38 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00333333"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00000000"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <color rgb="00000000"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Consolas"/>
-      <b val="1"/>
-      <color rgb="00003366"/>
-      <sz val="9"/>
+      <color rgb="00002060"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
   <fills count="6">
@@ -73,14 +72,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3D59"/>
-        <bgColor rgb="001E3D59"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002B5B84"/>
-        <bgColor rgb="002B5B84"/>
+        <fgColor rgb="002F5597"/>
+        <bgColor rgb="002F5597"/>
       </patternFill>
     </fill>
     <fill>
@@ -91,8 +90,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5F8"/>
-        <bgColor rgb="00F2F5F8"/>
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,16 +105,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
@@ -517,33 +516,33 @@
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>F1 · INVENTARIO DE ARTEFACTOS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Registre artefactos existentes o planificados; el estado debe reflejar la realidad del repositorio.</t>
+          <t>Registre artefactos existentes o planificados; el estado debe reflejar la realidad.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ID</t>
@@ -590,7 +589,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>A-01</t>
@@ -603,7 +602,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Descripción del problema, usuarios, objetivos y límites del sistema</t>
+          <t>Descripción del problema, usuarios y límites</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -623,7 +622,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -633,11 +632,11 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Base conceptual completa</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
+          <t>Documento base del alcance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>A-02</t>
@@ -650,7 +649,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Seguridad, rendimiento, usabilidad (ISO/IEC 25010 RC-01 a RC-10)</t>
+          <t>Seguridad, rendimiento, usabilidad, etc.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -670,7 +669,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -680,11 +679,11 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Actualizado mediante cambio CH-001 (métrica p99)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+          <t>Ajustado por cambio CH-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>A-03</t>
@@ -697,7 +696,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Componentes, tecnologías y relaciones cliente-servidor modulares</t>
+          <t>Componentes, tecnologías y relaciones</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -717,7 +716,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -731,7 +730,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>A-04</t>
@@ -744,7 +743,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>60+ casos de prueba con datos, entradas y resultados esperados</t>
+          <t>Casos, datos y resultados esperados</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -764,7 +763,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -774,11 +773,11 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Cubre CP-AUT, CP-MAT, CP-PAG, CP-REP, CP-NF</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
+          <t>Casos unitarios y de sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>A-05</t>
@@ -791,7 +790,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Aplicación web React y API REST Node.js + Express con reglas puras</t>
+          <t>Código de la aplicación</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -811,7 +810,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -821,11 +820,11 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Reglas y tests Jest 100% listos; vistas en curso</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
+          <t>Reglas puras y pruebas unitarias Jest</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>A-06</t>
@@ -838,7 +837,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Variables de entorno para API, JWT, BD PostgreSQL y SMTP</t>
+          <t>Variables de entorno para API y servicios</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -858,7 +857,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -868,11 +867,11 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Plantilla limpia sin claves privadas reales</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
+          <t>Variables de entorno de ejemplo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>A-07</t>
@@ -885,7 +884,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Instrucciones de instalación, despliegue y ejecución de pruebas</t>
+          <t>Instrucciones de instalación y ejecución</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -905,7 +904,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -915,7 +914,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Guía oficial para evaluadores y colaboradores</t>
+          <t>Documentación de uso</t>
         </is>
       </c>
     </row>
@@ -937,25 +936,25 @@
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="39" customWidth="1" min="8" max="8"/>
     <col width="43" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>F2 · REGISTRO DE VERSIONES</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Registre commits reales del repositorio. No invente hashes: copie el identificador mostrado por Git.</t>
@@ -963,7 +962,7 @@
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>N.º</t>
@@ -1010,7 +1009,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>1</t>
@@ -1018,7 +1017,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>28/10/2026 13:37</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -1043,21 +1042,21 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Registrar la estructura inicial del repositorio y plantillas</t>
+          <t>Registrar estructura inicial del proyecto</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>git status y verificación visual</t>
+          <t>git status y revision de archivos</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Versión inicial (A-06, A-07)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
+          <t>Versión inicial</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>2</t>
@@ -1065,7 +1064,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>28/10/2026 13:37</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -1090,12 +1089,12 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Definir objetivos, alcance, usuarios y requisitos ISO 25010</t>
+          <t>Formalizar alcance y requisitos de calidad</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Revisión documental y git status</t>
+          <t>Revision de documentos y git status</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -1104,7 +1103,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>3</t>
@@ -1112,7 +1111,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>28/10/2026 13:37</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -1132,17 +1131,17 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md; docs/04-casos-prueba.md; docs/Diagrama_arquitectura.drawio.png</t>
+          <t>docs/03-arquitectura.md; docs/04-casos-prueba.md; Diagrama_arquitectura.drawio.png</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Documentar capas de arquitectura y suite de 60+ casos de prueba</t>
+          <t>Documentar componentes y casos de prueba</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Verificación de diagramas y rutas</t>
+          <t>Verificacion de diagramas y rutas</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1151,7 +1150,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>4</t>
@@ -1159,7 +1158,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>28/10/2026 13:37</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -1179,17 +1178,17 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>src/backend/*; src/frontend/*</t>
+          <t>src/</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Incorporar código ejecutable con reglas puras de matrícula y React</t>
+          <t>Incorporar codigo fuente ejecutable y pruebas</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Ejecución de suite Jest (npm test)</t>
+          <t>Ejecucion de pruebas Jest (npm test)</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
@@ -1198,7 +1197,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>5</t>
@@ -1206,7 +1205,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>28/10/2026 13:39</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -1231,7 +1230,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Detallar créditos excedidos al estudiante y métrica p99 en RC-01</t>
+          <t>Detallar error en limite de creditos y ajustar metrica</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1263,27 +1262,27 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>F3 · REGISTRO DE CAMBIOS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Use para documentar la modificación práctica y preparar la gestión formal de cambios de la semana 11.</t>
@@ -1291,7 +1290,7 @@
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ID cambio</t>
@@ -1348,7 +1347,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>CH-001</t>
@@ -1361,22 +1360,22 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Registros Académicos / Equipo</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Mejorar mensaje de error en límite de créditos detallando total solicitado y precisar p99 en RC-01</t>
+          <t>Ajustar mensaje de error en limite de creditos detallando total solicitado y precisar metrica p99 en RC-01</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Evitar confusión del estudiante al exceder 22 créditos y definir umbral p99 bajo carga pico</t>
+          <t>Aclarar al estudiante la razon del rechazo al matricular mas de 22 creditos y fijar metrica en alta demanda</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>RC-01 (Rendimiento) y RC-04 / RF-04 (Límite créditos)</t>
+          <t>RC-01 (Rendimiento) y RC-04 / RF-04 (Limite de creditos)</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -1386,12 +1385,12 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Bajo: mejora la claridad del mensaje sin afectar contratos de API ni BD</t>
+          <t>Bajo. No altera contratos de API ni base de datos</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Pruebas unitarias Jest (rules.test.js) y git diff HEAD~1 HEAD</t>
+          <t>Pruebas unitarias Jest y git diff HEAD~1 HEAD</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -1401,7 +1400,7 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Aprobado por Miguel (Líder técnico)</t>
+          <t>Miguel Gronert</t>
         </is>
       </c>
     </row>
@@ -1423,24 +1422,24 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>F4 · MATRIZ DE TRAZABILIDAD</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Relacione requisitos con artefactos, pruebas y versiones cuando exista información suficiente.</t>
@@ -1448,7 +1447,7 @@
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ID Requisito</t>
@@ -1490,7 +1489,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>RC-01</t>
@@ -1503,12 +1502,12 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Rendimiento: 2000 concurrentes, 95% ops ≤3s, oferta ≤1.5s, p99 ≤4s</t>
+          <t>Rendimiento: 2000 concurrentes, 95% ops &lt;= 3s, oferta &lt;= 1.5s, p99 &lt;= 4s</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md (Caché Redis y PostgreSQL)</t>
+          <t>docs/03-arquitectura.md</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1532,7 +1531,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>RC-02</t>
@@ -1550,7 +1549,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md (Módulo Autenticación y Roles)</t>
+          <t>docs/03-arquitectura.md</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1574,7 +1573,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>RC-03</t>
@@ -1587,12 +1586,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Disponibilidad: ≥ 99.5 % durante periodo de matrícula</t>
+          <t>Disponibilidad: &gt;= 99.5 % durante periodo de matrícula</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md (Node.js stateless)</t>
+          <t>docs/03-arquitectura.md</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1616,7 +1615,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
+    <row r="8" ht="22" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>RC-04</t>
@@ -1629,12 +1628,12 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Integridad: 0 sobrecupos y transacciones atómicas</t>
+          <t>Integridad: 0 sobrecupos y operaciones transaccionales</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md (Módulo Matrícula)</t>
+          <t>docs/03-arquitectura.md</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1644,7 +1643,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>CP-MAT-08, 20, 21, CP-NF-02, 03</t>
+          <t>CP-MAT-08, 20, 21</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1658,7 +1657,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>RC-05</t>
@@ -1671,12 +1670,12 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Usabilidad: Matrícula ≤ 10 min, móvil (≥360px), WCAG 2.1 AA</t>
+          <t>Usabilidad: Matrícula en &lt;= 10 min, responsive móvil, WCAG 2.1 AA</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md (React SPA)</t>
+          <t>docs/03-arquitectura.md</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1686,7 +1685,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>CP-NF-06, 07, 08, 09</t>
+          <t>CP-NF-06, 07, 08</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -1700,7 +1699,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>RC-06</t>
@@ -1713,12 +1712,12 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Auditoría: Registro persistente de usuario, fecha/hora y acción</t>
+          <t>Auditoría: Registro de usuario, fecha/hora y acción en toda operación</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md (Módulo Auditoría)</t>
+          <t>docs/03-arquitectura.md</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -1742,7 +1741,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>RC-07</t>
@@ -1755,12 +1754,12 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Mantenibilidad: Pruebas unitarias ≥ 70% en reglas de negocio y Git</t>
+          <t>Mantenibilidad: Cobertura de pruebas unitarias &gt;= 70 % en reglas</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>docs/03-arquitectura.md (Diseño modular)</t>
+          <t>docs/03-arquitectura.md</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1780,11 +1779,11 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Cubierto 100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
+          <t>Cubierto</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>RF-01</t>
@@ -1826,7 +1825,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>RF-02</t>
@@ -1868,7 +1867,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
+    <row r="14" ht="22" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>RF-03</t>
@@ -1910,7 +1909,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>RF-04</t>
@@ -1923,7 +1922,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Control estricto de límite máximo de créditos (22 créditos)</t>
+          <t>Control del límite de créditos permitidos (22 créditos)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1952,7 +1951,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
+    <row r="16" ht="22" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>RF-05</t>
@@ -1994,7 +1993,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>RF-06</t>

</xml_diff>